<commit_message>
Update admin username to praveen and password to praveen1732@
</commit_message>
<xml_diff>
--- a/fun_questions.xlsx
+++ b/fun_questions.xlsx
@@ -962,7 +962,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G39"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -989,7 +989,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>13/9/2026, 6:54:16 pm</v>
+        <v>13/9/2026, 7:33:20 pm</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -1001,7 +1001,7 @@
         <v>AI Random Question</v>
       </c>
       <c r="E2" t="str">
-        <v>If exams disappeared tomorrow, what would you do first? 😂</v>
+        <v>Which of your friends would secretly become a college professor? 👨‍🏫</v>
       </c>
       <c r="F2" t="str">
         <v>Mathematics and Calculus</v>
@@ -1012,7 +1012,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>13/9/2026, 6:54:12 pm</v>
+        <v>13/9/2026, 7:33:20 pm</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -1035,7 +1035,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>13/9/2026, 6:54:12 pm</v>
+        <v>13/9/2026, 7:33:20 pm</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -1058,7 +1058,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>13/9/2026, 6:54:12 pm</v>
+        <v>13/9/2026, 7:33:20 pm</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -1081,7 +1081,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>13/9/2026, 6:54:12 pm</v>
+        <v>13/9/2026, 7:33:20 pm</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -1104,7 +1104,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>13/9/2026, 6:54:12 pm</v>
+        <v>13/9/2026, 7:33:20 pm</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -1127,7 +1127,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>13/9/2026, 6:54:12 pm</v>
+        <v>13/9/2026, 7:33:20 pm</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -1150,7 +1150,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>13/9/2026, 6:54:12 pm</v>
+        <v>13/9/2026, 7:33:20 pm</v>
       </c>
       <c r="B9">
         <v>1</v>
@@ -1173,7 +1173,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>13/9/2026, 6:54:12 pm</v>
+        <v>13/9/2026, 7:33:20 pm</v>
       </c>
       <c r="B10">
         <v>1</v>
@@ -1196,7 +1196,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>13/9/2026, 6:54:12 pm</v>
+        <v>13/9/2026, 7:33:20 pm</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -1219,7 +1219,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>13/9/2026, 6:54:12 pm</v>
+        <v>13/9/2026, 7:33:20 pm</v>
       </c>
       <c r="B12">
         <v>1</v>
@@ -1242,7 +1242,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>13/9/2026, 6:54:12 pm</v>
+        <v>13/9/2026, 7:33:20 pm</v>
       </c>
       <c r="B13">
         <v>1</v>
@@ -1265,7 +1265,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>13/9/2026, 6:54:12 pm</v>
+        <v>13/9/2026, 7:33:20 pm</v>
       </c>
       <c r="B14">
         <v>1</v>
@@ -1288,7 +1288,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>13/9/2026, 6:54:12 pm</v>
+        <v>13/9/2026, 7:33:20 pm</v>
       </c>
       <c r="B15">
         <v>1</v>
@@ -1311,7 +1311,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>13/9/2026, 6:54:12 pm</v>
+        <v>13/9/2026, 7:33:20 pm</v>
       </c>
       <c r="B16">
         <v>1</v>
@@ -1334,7 +1334,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>13/9/2026, 6:54:12 pm</v>
+        <v>13/9/2026, 7:33:20 pm</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -1357,7 +1357,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>13/9/2026, 6:53:31 pm</v>
+        <v>13/9/2026, 6:54:16 pm</v>
       </c>
       <c r="B18">
         <v>1</v>
@@ -1369,7 +1369,7 @@
         <v>AI Random Question</v>
       </c>
       <c r="E18" t="str">
-        <v>What is your all-time most-used emoji during exam week? 🧐</v>
+        <v>If exams disappeared tomorrow, what would you do first? 😂</v>
       </c>
       <c r="F18" t="str">
         <v>Mathematics and Calculus</v>
@@ -1380,7 +1380,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>13/9/2026, 6:53:17 pm</v>
+        <v>13/9/2026, 6:53:31 pm</v>
       </c>
       <c r="B19">
         <v>1</v>
@@ -1403,7 +1403,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>13/9/2026, 6:52:58 pm</v>
+        <v>13/9/2026, 6:53:17 pm</v>
       </c>
       <c r="B20">
         <v>1</v>
@@ -1415,7 +1415,7 @@
         <v>AI Random Question</v>
       </c>
       <c r="E20" t="str">
-        <v>If exams disappeared tomorrow, what would you do first? 😂</v>
+        <v>What is your all-time most-used emoji during exam week? 🧐</v>
       </c>
       <c r="F20" t="str">
         <v>Mathematics and Calculus</v>
@@ -1426,7 +1426,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>13/9/2026, 6:52:21 pm</v>
+        <v>13/9/2026, 6:52:58 pm</v>
       </c>
       <c r="B21">
         <v>1</v>
@@ -1449,25 +1449,25 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>13/9/2026, 6:41:44 pm</v>
+        <v>13/9/2026, 6:52:21 pm</v>
       </c>
       <c r="B22">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C22" t="str">
-        <v>praveen kumar</v>
+        <v>Alex Mercer</v>
       </c>
       <c r="D22" t="str">
-        <v>Squad Check-Up</v>
+        <v>AI Random Question</v>
       </c>
       <c r="E22" t="str">
-        <v>If your life were an anime/game/movie, what would its title be?</v>
+        <v>If exams disappeared tomorrow, what would you do first? 😂</v>
       </c>
       <c r="F22" t="str">
-        <v>solo leveling</v>
+        <v>Mathematics and Calculus</v>
       </c>
       <c r="G22" t="str">
-        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+        <v>💀 Mathematics catching stray arrows as usual! We will conquer it together!</v>
       </c>
     </row>
     <row r="23">
@@ -1484,10 +1484,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E23" t="str">
-        <v>If you had a completely free day tomorrow, what would you do?</v>
+        <v>If your life were an anime/game/movie, what would its title be?</v>
       </c>
       <c r="F23" t="str">
-        <v>non stop gaming</v>
+        <v>solo leveling</v>
       </c>
       <c r="G23" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1507,10 +1507,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E24" t="str">
-        <v>What is the funniest thing that happened in your college life?</v>
+        <v>If you had a completely free day tomorrow, what would you do?</v>
       </c>
       <c r="F24" t="str">
-        <v>play find the importer</v>
+        <v>non stop gaming</v>
       </c>
       <c r="G24" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1530,10 +1530,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E25" t="str">
-        <v>Who is your female best friend?</v>
+        <v>What is the funniest thing that happened in your college life?</v>
       </c>
       <c r="F25" t="str">
-        <v>pavithra</v>
+        <v>play find the importer</v>
       </c>
       <c r="G25" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1553,10 +1553,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E26" t="str">
-        <v>Who is your male best friend?</v>
+        <v>Who is your female best friend?</v>
       </c>
       <c r="F26" t="str">
-        <v>rupesh</v>
+        <v>pavithra</v>
       </c>
       <c r="G26" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1576,10 +1576,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E27" t="str">
-        <v>Do you have a funny or secret nickname?</v>
+        <v>Who is your male best friend?</v>
       </c>
       <c r="F27" t="str">
-        <v>chapri</v>
+        <v>rupesh</v>
       </c>
       <c r="G27" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1599,10 +1599,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E28" t="str">
-        <v>What's your favorite movie, anime, series, or game?</v>
+        <v>Do you have a funny or secret nickname?</v>
       </c>
       <c r="F28" t="str">
-        <v>attack on titan</v>
+        <v>chapri</v>
       </c>
       <c r="G28" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1622,10 +1622,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E29" t="str">
-        <v>Which friend would survive an exam with you?</v>
+        <v>What's your favorite movie, anime, series, or game?</v>
       </c>
       <c r="F29" t="str">
-        <v>sanjay</v>
+        <v>attack on titan</v>
       </c>
       <c r="G29" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1645,10 +1645,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E30" t="str">
-        <v>What's your favorite way to relax?</v>
+        <v>Which friend would survive an exam with you?</v>
       </c>
       <c r="F30" t="str">
-        <v>🎮 Gaming</v>
+        <v>sanjay</v>
       </c>
       <c r="G30" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1668,10 +1668,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E31" t="str">
-        <v>Which subject is your biggest enemy?</v>
+        <v>What's your favorite way to relax?</v>
       </c>
       <c r="F31" t="str">
-        <v>tamil</v>
+        <v>🎮 Gaming</v>
       </c>
       <c r="G31" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1691,10 +1691,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E32" t="str">
-        <v>Who is your study buddy?</v>
+        <v>Which subject is your biggest enemy?</v>
       </c>
       <c r="F32" t="str">
-        <v>sanjay</v>
+        <v>tamil</v>
       </c>
       <c r="G32" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1714,10 +1714,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E33" t="str">
-        <v>Who would you call when you're having a bad day?</v>
+        <v>Who is your study buddy?</v>
       </c>
       <c r="F33" t="str">
-        <v>myself</v>
+        <v>sanjay</v>
       </c>
       <c r="G33" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1737,10 +1737,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E34" t="str">
-        <v>Who do you text the most?</v>
+        <v>Who would you call when you're having a bad day?</v>
       </c>
       <c r="F34" t="str">
-        <v>pavithra</v>
+        <v>myself</v>
       </c>
       <c r="G34" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1760,10 +1760,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E35" t="str">
-        <v>Who makes you laugh the most?</v>
+        <v>Who do you text the most?</v>
       </c>
       <c r="F35" t="str">
-        <v>pk</v>
+        <v>pavithra</v>
       </c>
       <c r="G35" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1783,10 +1783,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E36" t="str">
-        <v>Who is your best friend?</v>
+        <v>Who makes you laugh the most?</v>
       </c>
       <c r="F36" t="str">
-        <v>sanjay</v>
+        <v>pk</v>
       </c>
       <c r="G36" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1794,30 +1794,30 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>13/9/2026, 6:37:12 pm</v>
+        <v>13/9/2026, 6:41:44 pm</v>
       </c>
       <c r="B37">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C37" t="str">
-        <v>Alex Mercer</v>
+        <v>praveen kumar</v>
       </c>
       <c r="D37" t="str">
-        <v>AI Random Question</v>
+        <v>Squad Check-Up</v>
       </c>
       <c r="E37" t="str">
-        <v>What is your most ridiculously productive time of day? ⏰</v>
+        <v>Who is your best friend?</v>
       </c>
       <c r="F37" t="str">
-        <v>Mathematics and Calculus</v>
+        <v>sanjay</v>
       </c>
       <c r="G37" t="str">
-        <v>💀 Mathematics catching stray arrows as usual! We will conquer it together!</v>
+        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>13/9/2026, 6:36:31 pm</v>
+        <v>13/9/2026, 6:37:12 pm</v>
       </c>
       <c r="B38">
         <v>1</v>
@@ -1829,7 +1829,7 @@
         <v>AI Random Question</v>
       </c>
       <c r="E38" t="str">
-        <v>Which fictional character would you choose as your study partner? 🦸</v>
+        <v>What is your most ridiculously productive time of day? ⏰</v>
       </c>
       <c r="F38" t="str">
         <v>Mathematics and Calculus</v>
@@ -1838,9 +1838,32 @@
         <v>💀 Mathematics catching stray arrows as usual! We will conquer it together!</v>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>13/9/2026, 6:36:31 pm</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Alex Mercer</v>
+      </c>
+      <c r="D39" t="str">
+        <v>AI Random Question</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Which fictional character would you choose as your study partner? 🦸</v>
+      </c>
+      <c r="F39" t="str">
+        <v>Mathematics and Calculus</v>
+      </c>
+      <c r="G39" t="str">
+        <v>💀 Mathematics catching stray arrows as usual! We will conquer it together!</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G39"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Remove public autofill buttons, obscure passwords in docs, and add secure Change Password feature
</commit_message>
<xml_diff>
--- a/fun_questions.xlsx
+++ b/fun_questions.xlsx
@@ -962,7 +962,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G40"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -989,7 +989,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>13/9/2026, 7:33:20 pm</v>
+        <v>13/9/2026, 7:39:09 pm</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -1001,7 +1001,7 @@
         <v>AI Random Question</v>
       </c>
       <c r="E2" t="str">
-        <v>Which of your friends would secretly become a college professor? 👨‍🏫</v>
+        <v>What is your all-time most-used emoji during exam week? 🧐</v>
       </c>
       <c r="F2" t="str">
         <v>Mathematics and Calculus</v>
@@ -1012,7 +1012,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>13/9/2026, 7:33:20 pm</v>
+        <v>13/9/2026, 7:39:08 pm</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -1035,7 +1035,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>13/9/2026, 7:33:20 pm</v>
+        <v>13/9/2026, 7:39:08 pm</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -1058,7 +1058,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>13/9/2026, 7:33:20 pm</v>
+        <v>13/9/2026, 7:39:08 pm</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -1081,7 +1081,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>13/9/2026, 7:33:20 pm</v>
+        <v>13/9/2026, 7:39:08 pm</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -1104,7 +1104,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>13/9/2026, 7:33:20 pm</v>
+        <v>13/9/2026, 7:39:08 pm</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -1127,7 +1127,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>13/9/2026, 7:33:20 pm</v>
+        <v>13/9/2026, 7:39:08 pm</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -1150,7 +1150,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>13/9/2026, 7:33:20 pm</v>
+        <v>13/9/2026, 7:39:08 pm</v>
       </c>
       <c r="B9">
         <v>1</v>
@@ -1173,7 +1173,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>13/9/2026, 7:33:20 pm</v>
+        <v>13/9/2026, 7:39:08 pm</v>
       </c>
       <c r="B10">
         <v>1</v>
@@ -1196,7 +1196,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>13/9/2026, 7:33:20 pm</v>
+        <v>13/9/2026, 7:39:08 pm</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -1219,7 +1219,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>13/9/2026, 7:33:20 pm</v>
+        <v>13/9/2026, 7:39:08 pm</v>
       </c>
       <c r="B12">
         <v>1</v>
@@ -1242,7 +1242,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>13/9/2026, 7:33:20 pm</v>
+        <v>13/9/2026, 7:39:08 pm</v>
       </c>
       <c r="B13">
         <v>1</v>
@@ -1265,7 +1265,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>13/9/2026, 7:33:20 pm</v>
+        <v>13/9/2026, 7:39:08 pm</v>
       </c>
       <c r="B14">
         <v>1</v>
@@ -1288,7 +1288,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>13/9/2026, 7:33:20 pm</v>
+        <v>13/9/2026, 7:39:08 pm</v>
       </c>
       <c r="B15">
         <v>1</v>
@@ -1311,7 +1311,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>13/9/2026, 7:33:20 pm</v>
+        <v>13/9/2026, 7:39:08 pm</v>
       </c>
       <c r="B16">
         <v>1</v>
@@ -1334,7 +1334,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>13/9/2026, 7:33:20 pm</v>
+        <v>13/9/2026, 7:39:08 pm</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -1357,7 +1357,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>13/9/2026, 6:54:16 pm</v>
+        <v>13/9/2026, 7:33:20 pm</v>
       </c>
       <c r="B18">
         <v>1</v>
@@ -1369,7 +1369,7 @@
         <v>AI Random Question</v>
       </c>
       <c r="E18" t="str">
-        <v>If exams disappeared tomorrow, what would you do first? 😂</v>
+        <v>Which of your friends would secretly become a college professor? 👨‍🏫</v>
       </c>
       <c r="F18" t="str">
         <v>Mathematics and Calculus</v>
@@ -1380,7 +1380,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>13/9/2026, 6:53:31 pm</v>
+        <v>13/9/2026, 6:54:16 pm</v>
       </c>
       <c r="B19">
         <v>1</v>
@@ -1392,7 +1392,7 @@
         <v>AI Random Question</v>
       </c>
       <c r="E19" t="str">
-        <v>What is your all-time most-used emoji during exam week? 🧐</v>
+        <v>If exams disappeared tomorrow, what would you do first? 😂</v>
       </c>
       <c r="F19" t="str">
         <v>Mathematics and Calculus</v>
@@ -1403,7 +1403,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>13/9/2026, 6:53:17 pm</v>
+        <v>13/9/2026, 6:53:31 pm</v>
       </c>
       <c r="B20">
         <v>1</v>
@@ -1426,7 +1426,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>13/9/2026, 6:52:58 pm</v>
+        <v>13/9/2026, 6:53:17 pm</v>
       </c>
       <c r="B21">
         <v>1</v>
@@ -1438,7 +1438,7 @@
         <v>AI Random Question</v>
       </c>
       <c r="E21" t="str">
-        <v>If exams disappeared tomorrow, what would you do first? 😂</v>
+        <v>What is your all-time most-used emoji during exam week? 🧐</v>
       </c>
       <c r="F21" t="str">
         <v>Mathematics and Calculus</v>
@@ -1449,7 +1449,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>13/9/2026, 6:52:21 pm</v>
+        <v>13/9/2026, 6:52:58 pm</v>
       </c>
       <c r="B22">
         <v>1</v>
@@ -1472,25 +1472,25 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>13/9/2026, 6:41:44 pm</v>
+        <v>13/9/2026, 6:52:21 pm</v>
       </c>
       <c r="B23">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C23" t="str">
-        <v>praveen kumar</v>
+        <v>Alex Mercer</v>
       </c>
       <c r="D23" t="str">
-        <v>Squad Check-Up</v>
+        <v>AI Random Question</v>
       </c>
       <c r="E23" t="str">
-        <v>If your life were an anime/game/movie, what would its title be?</v>
+        <v>If exams disappeared tomorrow, what would you do first? 😂</v>
       </c>
       <c r="F23" t="str">
-        <v>solo leveling</v>
+        <v>Mathematics and Calculus</v>
       </c>
       <c r="G23" t="str">
-        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+        <v>💀 Mathematics catching stray arrows as usual! We will conquer it together!</v>
       </c>
     </row>
     <row r="24">
@@ -1507,10 +1507,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E24" t="str">
-        <v>If you had a completely free day tomorrow, what would you do?</v>
+        <v>If your life were an anime/game/movie, what would its title be?</v>
       </c>
       <c r="F24" t="str">
-        <v>non stop gaming</v>
+        <v>solo leveling</v>
       </c>
       <c r="G24" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1530,10 +1530,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E25" t="str">
-        <v>What is the funniest thing that happened in your college life?</v>
+        <v>If you had a completely free day tomorrow, what would you do?</v>
       </c>
       <c r="F25" t="str">
-        <v>play find the importer</v>
+        <v>non stop gaming</v>
       </c>
       <c r="G25" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1553,10 +1553,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E26" t="str">
-        <v>Who is your female best friend?</v>
+        <v>What is the funniest thing that happened in your college life?</v>
       </c>
       <c r="F26" t="str">
-        <v>pavithra</v>
+        <v>play find the importer</v>
       </c>
       <c r="G26" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1576,10 +1576,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E27" t="str">
-        <v>Who is your male best friend?</v>
+        <v>Who is your female best friend?</v>
       </c>
       <c r="F27" t="str">
-        <v>rupesh</v>
+        <v>pavithra</v>
       </c>
       <c r="G27" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1599,10 +1599,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E28" t="str">
-        <v>Do you have a funny or secret nickname?</v>
+        <v>Who is your male best friend?</v>
       </c>
       <c r="F28" t="str">
-        <v>chapri</v>
+        <v>rupesh</v>
       </c>
       <c r="G28" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1622,10 +1622,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E29" t="str">
-        <v>What's your favorite movie, anime, series, or game?</v>
+        <v>Do you have a funny or secret nickname?</v>
       </c>
       <c r="F29" t="str">
-        <v>attack on titan</v>
+        <v>chapri</v>
       </c>
       <c r="G29" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1645,10 +1645,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E30" t="str">
-        <v>Which friend would survive an exam with you?</v>
+        <v>What's your favorite movie, anime, series, or game?</v>
       </c>
       <c r="F30" t="str">
-        <v>sanjay</v>
+        <v>attack on titan</v>
       </c>
       <c r="G30" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1668,10 +1668,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E31" t="str">
-        <v>What's your favorite way to relax?</v>
+        <v>Which friend would survive an exam with you?</v>
       </c>
       <c r="F31" t="str">
-        <v>🎮 Gaming</v>
+        <v>sanjay</v>
       </c>
       <c r="G31" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1691,10 +1691,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E32" t="str">
-        <v>Which subject is your biggest enemy?</v>
+        <v>What's your favorite way to relax?</v>
       </c>
       <c r="F32" t="str">
-        <v>tamil</v>
+        <v>🎮 Gaming</v>
       </c>
       <c r="G32" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1714,10 +1714,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E33" t="str">
-        <v>Who is your study buddy?</v>
+        <v>Which subject is your biggest enemy?</v>
       </c>
       <c r="F33" t="str">
-        <v>sanjay</v>
+        <v>tamil</v>
       </c>
       <c r="G33" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1737,10 +1737,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E34" t="str">
-        <v>Who would you call when you're having a bad day?</v>
+        <v>Who is your study buddy?</v>
       </c>
       <c r="F34" t="str">
-        <v>myself</v>
+        <v>sanjay</v>
       </c>
       <c r="G34" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1760,10 +1760,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E35" t="str">
-        <v>Who do you text the most?</v>
+        <v>Who would you call when you're having a bad day?</v>
       </c>
       <c r="F35" t="str">
-        <v>pavithra</v>
+        <v>myself</v>
       </c>
       <c r="G35" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1783,10 +1783,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E36" t="str">
-        <v>Who makes you laugh the most?</v>
+        <v>Who do you text the most?</v>
       </c>
       <c r="F36" t="str">
-        <v>pk</v>
+        <v>pavithra</v>
       </c>
       <c r="G36" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1806,10 +1806,10 @@
         <v>Squad Check-Up</v>
       </c>
       <c r="E37" t="str">
-        <v>Who is your best friend?</v>
+        <v>Who makes you laugh the most?</v>
       </c>
       <c r="F37" t="str">
-        <v>sanjay</v>
+        <v>pk</v>
       </c>
       <c r="G37" t="str">
         <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
@@ -1817,30 +1817,30 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>13/9/2026, 6:37:12 pm</v>
+        <v>13/9/2026, 6:41:44 pm</v>
       </c>
       <c r="B38">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C38" t="str">
-        <v>Alex Mercer</v>
+        <v>praveen kumar</v>
       </c>
       <c r="D38" t="str">
-        <v>AI Random Question</v>
+        <v>Squad Check-Up</v>
       </c>
       <c r="E38" t="str">
-        <v>What is your most ridiculously productive time of day? ⏰</v>
+        <v>Who is your best friend?</v>
       </c>
       <c r="F38" t="str">
-        <v>Mathematics and Calculus</v>
+        <v>sanjay</v>
       </c>
       <c r="G38" t="str">
-        <v>💀 Mathematics catching stray arrows as usual! We will conquer it together!</v>
+        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>13/9/2026, 6:36:31 pm</v>
+        <v>13/9/2026, 6:37:12 pm</v>
       </c>
       <c r="B39">
         <v>1</v>
@@ -1852,7 +1852,7 @@
         <v>AI Random Question</v>
       </c>
       <c r="E39" t="str">
-        <v>Which fictional character would you choose as your study partner? 🦸</v>
+        <v>What is your most ridiculously productive time of day? ⏰</v>
       </c>
       <c r="F39" t="str">
         <v>Mathematics and Calculus</v>
@@ -1861,9 +1861,32 @@
         <v>💀 Mathematics catching stray arrows as usual! We will conquer it together!</v>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>13/9/2026, 6:36:31 pm</v>
+      </c>
+      <c r="B40">
+        <v>1</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Alex Mercer</v>
+      </c>
+      <c r="D40" t="str">
+        <v>AI Random Question</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Which fictional character would you choose as your study partner? 🦸</v>
+      </c>
+      <c r="F40" t="str">
+        <v>Mathematics and Calculus</v>
+      </c>
+      <c r="G40" t="str">
+        <v>💀 Mathematics catching stray arrows as usual! We will conquer it together!</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G39"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G40"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update admin credentials for praveen with email, password, phone contact, and profile schema
</commit_message>
<xml_diff>
--- a/fun_questions.xlsx
+++ b/fun_questions.xlsx
@@ -962,7 +962,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G89"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -989,19 +989,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>13/9/2026, 7:39:09 pm</v>
+        <v>13/9/2026, 8:50:30 pm</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="C2" t="str">
-        <v>Alex Mercer</v>
+        <v>Test Student</v>
       </c>
       <c r="D2" t="str">
         <v>AI Random Question</v>
       </c>
       <c r="E2" t="str">
-        <v>What is your all-time most-used emoji during exam week? 🧐</v>
+        <v>What is the weirdest place you have ever studied for an exam? 🗺️</v>
       </c>
       <c r="F2" t="str">
         <v>Mathematics and Calculus</v>
@@ -1012,13 +1012,13 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>13/9/2026, 7:39:08 pm</v>
+        <v>13/9/2026, 8:50:29 pm</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="C3" t="str">
-        <v>Alex Mercer</v>
+        <v>Test Student</v>
       </c>
       <c r="D3" t="str">
         <v>Squad Check-Up</v>
@@ -1035,13 +1035,13 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>13/9/2026, 7:39:08 pm</v>
+        <v>13/9/2026, 8:50:29 pm</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="C4" t="str">
-        <v>Alex Mercer</v>
+        <v>Test Student</v>
       </c>
       <c r="D4" t="str">
         <v>Squad Check-Up</v>
@@ -1058,13 +1058,13 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>13/9/2026, 7:39:08 pm</v>
+        <v>13/9/2026, 8:50:29 pm</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="C5" t="str">
-        <v>Alex Mercer</v>
+        <v>Test Student</v>
       </c>
       <c r="D5" t="str">
         <v>Squad Check-Up</v>
@@ -1081,13 +1081,13 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>13/9/2026, 7:39:08 pm</v>
+        <v>13/9/2026, 8:50:29 pm</v>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="C6" t="str">
-        <v>Alex Mercer</v>
+        <v>Test Student</v>
       </c>
       <c r="D6" t="str">
         <v>Squad Check-Up</v>
@@ -1104,13 +1104,13 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>13/9/2026, 7:39:08 pm</v>
+        <v>13/9/2026, 8:50:29 pm</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="C7" t="str">
-        <v>Alex Mercer</v>
+        <v>Test Student</v>
       </c>
       <c r="D7" t="str">
         <v>Squad Check-Up</v>
@@ -1127,13 +1127,13 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>13/9/2026, 7:39:08 pm</v>
+        <v>13/9/2026, 8:50:29 pm</v>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="C8" t="str">
-        <v>Alex Mercer</v>
+        <v>Test Student</v>
       </c>
       <c r="D8" t="str">
         <v>Squad Check-Up</v>
@@ -1150,13 +1150,13 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>13/9/2026, 7:39:08 pm</v>
+        <v>13/9/2026, 8:50:29 pm</v>
       </c>
       <c r="B9">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="C9" t="str">
-        <v>Alex Mercer</v>
+        <v>Test Student</v>
       </c>
       <c r="D9" t="str">
         <v>Squad Check-Up</v>
@@ -1173,13 +1173,13 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>13/9/2026, 7:39:08 pm</v>
+        <v>13/9/2026, 8:50:29 pm</v>
       </c>
       <c r="B10">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="C10" t="str">
-        <v>Alex Mercer</v>
+        <v>Test Student</v>
       </c>
       <c r="D10" t="str">
         <v>Squad Check-Up</v>
@@ -1196,13 +1196,13 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>13/9/2026, 7:39:08 pm</v>
+        <v>13/9/2026, 8:50:29 pm</v>
       </c>
       <c r="B11">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="C11" t="str">
-        <v>Alex Mercer</v>
+        <v>Test Student</v>
       </c>
       <c r="D11" t="str">
         <v>Squad Check-Up</v>
@@ -1219,13 +1219,13 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>13/9/2026, 7:39:08 pm</v>
+        <v>13/9/2026, 8:50:29 pm</v>
       </c>
       <c r="B12">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="C12" t="str">
-        <v>Alex Mercer</v>
+        <v>Test Student</v>
       </c>
       <c r="D12" t="str">
         <v>Squad Check-Up</v>
@@ -1242,13 +1242,13 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>13/9/2026, 7:39:08 pm</v>
+        <v>13/9/2026, 8:50:29 pm</v>
       </c>
       <c r="B13">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="C13" t="str">
-        <v>Alex Mercer</v>
+        <v>Test Student</v>
       </c>
       <c r="D13" t="str">
         <v>Squad Check-Up</v>
@@ -1265,13 +1265,13 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>13/9/2026, 7:39:08 pm</v>
+        <v>13/9/2026, 8:50:29 pm</v>
       </c>
       <c r="B14">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="C14" t="str">
-        <v>Alex Mercer</v>
+        <v>Test Student</v>
       </c>
       <c r="D14" t="str">
         <v>Squad Check-Up</v>
@@ -1288,13 +1288,13 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>13/9/2026, 7:39:08 pm</v>
+        <v>13/9/2026, 8:50:29 pm</v>
       </c>
       <c r="B15">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="C15" t="str">
-        <v>Alex Mercer</v>
+        <v>Test Student</v>
       </c>
       <c r="D15" t="str">
         <v>Squad Check-Up</v>
@@ -1311,13 +1311,13 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>13/9/2026, 7:39:08 pm</v>
+        <v>13/9/2026, 8:50:29 pm</v>
       </c>
       <c r="B16">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="C16" t="str">
-        <v>Alex Mercer</v>
+        <v>Test Student</v>
       </c>
       <c r="D16" t="str">
         <v>Squad Check-Up</v>
@@ -1334,13 +1334,13 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>13/9/2026, 7:39:08 pm</v>
+        <v>13/9/2026, 8:50:29 pm</v>
       </c>
       <c r="B17">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="C17" t="str">
-        <v>Alex Mercer</v>
+        <v>Test Student</v>
       </c>
       <c r="D17" t="str">
         <v>Squad Check-Up</v>
@@ -1357,13 +1357,13 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>13/9/2026, 7:33:20 pm</v>
+        <v>13/9/2026, 8:36:03 pm</v>
       </c>
       <c r="B18">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="C18" t="str">
-        <v>Alex Mercer</v>
+        <v>Test Student</v>
       </c>
       <c r="D18" t="str">
         <v>AI Random Question</v>
@@ -1380,513 +1380,1640 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>13/9/2026, 6:54:16 pm</v>
+        <v>13/9/2026, 8:36:02 pm</v>
       </c>
       <c r="B19">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="C19" t="str">
-        <v>Alex Mercer</v>
+        <v>Test Student</v>
       </c>
       <c r="D19" t="str">
-        <v>AI Random Question</v>
+        <v>Squad Check-Up</v>
       </c>
       <c r="E19" t="str">
-        <v>If exams disappeared tomorrow, what would you do first? 😂</v>
+        <v>If your life were an anime/game/movie, what would its title be?</v>
       </c>
       <c r="F19" t="str">
-        <v>Mathematics and Calculus</v>
+        <v>Solo Leveling: The Finals Arc ⚔️</v>
       </c>
       <c r="G19" t="str">
-        <v>💀 Mathematics catching stray arrows as usual! We will conquer it together!</v>
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>13/9/2026, 6:53:31 pm</v>
+        <v>13/9/2026, 8:36:02 pm</v>
       </c>
       <c r="B20">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="C20" t="str">
-        <v>Alex Mercer</v>
+        <v>Test Student</v>
       </c>
       <c r="D20" t="str">
-        <v>AI Random Question</v>
+        <v>Squad Check-Up</v>
       </c>
       <c r="E20" t="str">
-        <v>What is your all-time most-used emoji during exam week? 🧐</v>
+        <v>If you had a completely free day tomorrow, what would you do?</v>
       </c>
       <c r="F20" t="str">
-        <v>Mathematics and Calculus</v>
+        <v>Sleep for 12 hours straight then binge anime 🍿</v>
       </c>
       <c r="G20" t="str">
-        <v>💀 Mathematics catching stray arrows as usual! We will conquer it together!</v>
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>13/9/2026, 6:53:17 pm</v>
+        <v>13/9/2026, 8:36:02 pm</v>
       </c>
       <c r="B21">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="C21" t="str">
-        <v>Alex Mercer</v>
+        <v>Test Student</v>
       </c>
       <c r="D21" t="str">
-        <v>AI Random Question</v>
+        <v>Squad Check-Up</v>
       </c>
       <c r="E21" t="str">
-        <v>What is your all-time most-used emoji during exam week? 🧐</v>
+        <v>What is the funniest thing that happened in your college life?</v>
       </c>
       <c r="F21" t="str">
-        <v>Mathematics and Calculus</v>
+        <v>Professor caught us playing games in the front row 😂</v>
       </c>
       <c r="G21" t="str">
-        <v>💀 Mathematics catching stray arrows as usual! We will conquer it together!</v>
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>13/9/2026, 6:52:58 pm</v>
+        <v>13/9/2026, 8:36:02 pm</v>
       </c>
       <c r="B22">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="C22" t="str">
-        <v>Alex Mercer</v>
+        <v>Test Student</v>
       </c>
       <c r="D22" t="str">
-        <v>AI Random Question</v>
+        <v>Squad Check-Up</v>
       </c>
       <c r="E22" t="str">
-        <v>If exams disappeared tomorrow, what would you do first? 😂</v>
+        <v>Who is your female best friend?</v>
       </c>
       <c r="F22" t="str">
-        <v>Mathematics and Calculus</v>
+        <v>Priya</v>
       </c>
       <c r="G22" t="str">
-        <v>💀 Mathematics catching stray arrows as usual! We will conquer it together!</v>
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>13/9/2026, 6:52:21 pm</v>
+        <v>13/9/2026, 8:36:02 pm</v>
       </c>
       <c r="B23">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="C23" t="str">
-        <v>Alex Mercer</v>
+        <v>Test Student</v>
       </c>
       <c r="D23" t="str">
-        <v>AI Random Question</v>
+        <v>Squad Check-Up</v>
       </c>
       <c r="E23" t="str">
-        <v>If exams disappeared tomorrow, what would you do first? 😂</v>
+        <v>Who is your male best friend?</v>
       </c>
       <c r="F23" t="str">
-        <v>Mathematics and Calculus</v>
+        <v>Rahul</v>
       </c>
       <c r="G23" t="str">
-        <v>💀 Mathematics catching stray arrows as usual! We will conquer it together!</v>
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>13/9/2026, 6:41:44 pm</v>
+        <v>13/9/2026, 8:36:02 pm</v>
       </c>
       <c r="B24">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="C24" t="str">
-        <v>praveen kumar</v>
+        <v>Test Student</v>
       </c>
       <c r="D24" t="str">
         <v>Squad Check-Up</v>
       </c>
       <c r="E24" t="str">
-        <v>If your life were an anime/game/movie, what would its title be?</v>
+        <v>Do you have a funny or secret nickname?</v>
       </c>
       <c r="F24" t="str">
-        <v>solo leveling</v>
+        <v>Rocky</v>
       </c>
       <c r="G24" t="str">
-        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>13/9/2026, 6:41:44 pm</v>
+        <v>13/9/2026, 8:36:02 pm</v>
       </c>
       <c r="B25">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="C25" t="str">
-        <v>praveen kumar</v>
+        <v>Test Student</v>
       </c>
       <c r="D25" t="str">
         <v>Squad Check-Up</v>
       </c>
       <c r="E25" t="str">
-        <v>If you had a completely free day tomorrow, what would you do?</v>
+        <v>What's your favorite movie, anime, series, or game?</v>
       </c>
       <c r="F25" t="str">
-        <v>non stop gaming</v>
+        <v>Interstellar</v>
       </c>
       <c r="G25" t="str">
-        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>13/9/2026, 6:41:44 pm</v>
+        <v>13/9/2026, 8:36:02 pm</v>
       </c>
       <c r="B26">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="C26" t="str">
-        <v>praveen kumar</v>
+        <v>Test Student</v>
       </c>
       <c r="D26" t="str">
         <v>Squad Check-Up</v>
       </c>
       <c r="E26" t="str">
-        <v>What is the funniest thing that happened in your college life?</v>
+        <v>Which friend would survive an exam with you?</v>
       </c>
       <c r="F26" t="str">
-        <v>play find the importer</v>
+        <v>Arun</v>
       </c>
       <c r="G26" t="str">
-        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>13/9/2026, 6:41:44 pm</v>
+        <v>13/9/2026, 8:36:02 pm</v>
       </c>
       <c r="B27">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="C27" t="str">
-        <v>praveen kumar</v>
+        <v>Test Student</v>
       </c>
       <c r="D27" t="str">
         <v>Squad Check-Up</v>
       </c>
       <c r="E27" t="str">
-        <v>Who is your female best friend?</v>
+        <v>What's your favorite way to relax?</v>
       </c>
       <c r="F27" t="str">
-        <v>pavithra</v>
+        <v>🎮 Gaming, ▶️ YouTube</v>
       </c>
       <c r="G27" t="str">
-        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>13/9/2026, 6:41:44 pm</v>
+        <v>13/9/2026, 8:36:02 pm</v>
       </c>
       <c r="B28">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="C28" t="str">
-        <v>praveen kumar</v>
+        <v>Test Student</v>
       </c>
       <c r="D28" t="str">
         <v>Squad Check-Up</v>
       </c>
       <c r="E28" t="str">
-        <v>Who is your male best friend?</v>
+        <v>Which subject is your biggest enemy?</v>
       </c>
       <c r="F28" t="str">
-        <v>rupesh</v>
+        <v>Mathematics</v>
       </c>
       <c r="G28" t="str">
-        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>13/9/2026, 6:41:44 pm</v>
+        <v>13/9/2026, 8:36:02 pm</v>
       </c>
       <c r="B29">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="C29" t="str">
-        <v>praveen kumar</v>
+        <v>Test Student</v>
       </c>
       <c r="D29" t="str">
         <v>Squad Check-Up</v>
       </c>
       <c r="E29" t="str">
-        <v>Do you have a funny or secret nickname?</v>
+        <v>Who is your study buddy?</v>
       </c>
       <c r="F29" t="str">
-        <v>chapri</v>
+        <v>Arun</v>
       </c>
       <c r="G29" t="str">
-        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>13/9/2026, 6:41:44 pm</v>
+        <v>13/9/2026, 8:36:02 pm</v>
       </c>
       <c r="B30">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="C30" t="str">
-        <v>praveen kumar</v>
+        <v>Test Student</v>
       </c>
       <c r="D30" t="str">
         <v>Squad Check-Up</v>
       </c>
       <c r="E30" t="str">
-        <v>What's your favorite movie, anime, series, or game?</v>
+        <v>Who would you call when you're having a bad day?</v>
       </c>
       <c r="F30" t="str">
-        <v>attack on titan</v>
+        <v>Karthik</v>
       </c>
       <c r="G30" t="str">
-        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>13/9/2026, 6:41:44 pm</v>
+        <v>13/9/2026, 8:36:02 pm</v>
       </c>
       <c r="B31">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="C31" t="str">
-        <v>praveen kumar</v>
+        <v>Test Student</v>
       </c>
       <c r="D31" t="str">
         <v>Squad Check-Up</v>
       </c>
       <c r="E31" t="str">
-        <v>Which friend would survive an exam with you?</v>
+        <v>Who do you text the most?</v>
       </c>
       <c r="F31" t="str">
-        <v>sanjay</v>
+        <v>Arun</v>
       </c>
       <c r="G31" t="str">
-        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>13/9/2026, 6:41:44 pm</v>
+        <v>13/9/2026, 8:36:02 pm</v>
       </c>
       <c r="B32">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="C32" t="str">
-        <v>praveen kumar</v>
+        <v>Test Student</v>
       </c>
       <c r="D32" t="str">
         <v>Squad Check-Up</v>
       </c>
       <c r="E32" t="str">
-        <v>What's your favorite way to relax?</v>
+        <v>Who makes you laugh the most?</v>
       </c>
       <c r="F32" t="str">
-        <v>🎮 Gaming</v>
+        <v>Karthik</v>
       </c>
       <c r="G32" t="str">
-        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>13/9/2026, 6:41:44 pm</v>
+        <v>13/9/2026, 8:36:02 pm</v>
       </c>
       <c r="B33">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="C33" t="str">
-        <v>praveen kumar</v>
+        <v>Test Student</v>
       </c>
       <c r="D33" t="str">
         <v>Squad Check-Up</v>
       </c>
       <c r="E33" t="str">
-        <v>Which subject is your biggest enemy?</v>
+        <v>Who is your best friend?</v>
       </c>
       <c r="F33" t="str">
-        <v>tamil</v>
+        <v>Arun</v>
       </c>
       <c r="G33" t="str">
-        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>13/9/2026, 6:41:44 pm</v>
+        <v>13/9/2026, 8:33:58 pm</v>
       </c>
       <c r="B34">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="C34" t="str">
-        <v>praveen kumar</v>
+        <v>Test Student</v>
       </c>
       <c r="D34" t="str">
-        <v>Squad Check-Up</v>
+        <v>AI Random Question</v>
       </c>
       <c r="E34" t="str">
-        <v>Who is your study buddy?</v>
+        <v>What is your most ridiculously productive time of day? ⏰</v>
       </c>
       <c r="F34" t="str">
-        <v>sanjay</v>
+        <v>Mathematics and Calculus</v>
       </c>
       <c r="G34" t="str">
-        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+        <v>💀 Mathematics catching stray arrows as usual! We will conquer it together!</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>13/9/2026, 6:41:44 pm</v>
+        <v>13/9/2026, 8:33:57 pm</v>
       </c>
       <c r="B35">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="C35" t="str">
-        <v>praveen kumar</v>
+        <v>Test Student</v>
       </c>
       <c r="D35" t="str">
         <v>Squad Check-Up</v>
       </c>
       <c r="E35" t="str">
-        <v>Who would you call when you're having a bad day?</v>
+        <v>If your life were an anime/game/movie, what would its title be?</v>
       </c>
       <c r="F35" t="str">
-        <v>myself</v>
+        <v>Solo Leveling: The Finals Arc ⚔️</v>
       </c>
       <c r="G35" t="str">
-        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>13/9/2026, 6:41:44 pm</v>
+        <v>13/9/2026, 8:33:57 pm</v>
       </c>
       <c r="B36">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="C36" t="str">
-        <v>praveen kumar</v>
+        <v>Test Student</v>
       </c>
       <c r="D36" t="str">
         <v>Squad Check-Up</v>
       </c>
       <c r="E36" t="str">
-        <v>Who do you text the most?</v>
+        <v>If you had a completely free day tomorrow, what would you do?</v>
       </c>
       <c r="F36" t="str">
-        <v>pavithra</v>
+        <v>Sleep for 12 hours straight then binge anime 🍿</v>
       </c>
       <c r="G36" t="str">
-        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>13/9/2026, 6:41:44 pm</v>
+        <v>13/9/2026, 8:33:57 pm</v>
       </c>
       <c r="B37">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="C37" t="str">
-        <v>praveen kumar</v>
+        <v>Test Student</v>
       </c>
       <c r="D37" t="str">
         <v>Squad Check-Up</v>
       </c>
       <c r="E37" t="str">
-        <v>Who makes you laugh the most?</v>
+        <v>What is the funniest thing that happened in your college life?</v>
       </c>
       <c r="F37" t="str">
-        <v>pk</v>
+        <v>Professor caught us playing games in the front row 😂</v>
       </c>
       <c r="G37" t="str">
-        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>13/9/2026, 6:41:44 pm</v>
+        <v>13/9/2026, 8:33:57 pm</v>
       </c>
       <c r="B38">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="C38" t="str">
-        <v>praveen kumar</v>
+        <v>Test Student</v>
       </c>
       <c r="D38" t="str">
         <v>Squad Check-Up</v>
       </c>
       <c r="E38" t="str">
-        <v>Who is your best friend?</v>
+        <v>Who is your female best friend?</v>
       </c>
       <c r="F38" t="str">
-        <v>sanjay</v>
+        <v>Priya</v>
       </c>
       <c r="G38" t="str">
-        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>13/9/2026, 6:37:12 pm</v>
+        <v>13/9/2026, 8:33:57 pm</v>
       </c>
       <c r="B39">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="C39" t="str">
-        <v>Alex Mercer</v>
+        <v>Test Student</v>
       </c>
       <c r="D39" t="str">
-        <v>AI Random Question</v>
+        <v>Squad Check-Up</v>
       </c>
       <c r="E39" t="str">
-        <v>What is your most ridiculously productive time of day? ⏰</v>
+        <v>Who is your male best friend?</v>
       </c>
       <c r="F39" t="str">
-        <v>Mathematics and Calculus</v>
+        <v>Rahul</v>
       </c>
       <c r="G39" t="str">
-        <v>💀 Mathematics catching stray arrows as usual! We will conquer it together!</v>
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
+        <v>13/9/2026, 8:33:57 pm</v>
+      </c>
+      <c r="B40">
+        <v>24</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Test Student</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Do you have a funny or secret nickname?</v>
+      </c>
+      <c r="F40" t="str">
+        <v>Rocky</v>
+      </c>
+      <c r="G40" t="str">
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>13/9/2026, 8:33:57 pm</v>
+      </c>
+      <c r="B41">
+        <v>24</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Test Student</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E41" t="str">
+        <v>What's your favorite movie, anime, series, or game?</v>
+      </c>
+      <c r="F41" t="str">
+        <v>Interstellar</v>
+      </c>
+      <c r="G41" t="str">
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>13/9/2026, 8:33:57 pm</v>
+      </c>
+      <c r="B42">
+        <v>24</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Test Student</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Which friend would survive an exam with you?</v>
+      </c>
+      <c r="F42" t="str">
+        <v>Arun</v>
+      </c>
+      <c r="G42" t="str">
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>13/9/2026, 8:33:57 pm</v>
+      </c>
+      <c r="B43">
+        <v>24</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Test Student</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E43" t="str">
+        <v>What's your favorite way to relax?</v>
+      </c>
+      <c r="F43" t="str">
+        <v>🎮 Gaming, ▶️ YouTube</v>
+      </c>
+      <c r="G43" t="str">
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>13/9/2026, 8:33:57 pm</v>
+      </c>
+      <c r="B44">
+        <v>24</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Test Student</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E44" t="str">
+        <v>Which subject is your biggest enemy?</v>
+      </c>
+      <c r="F44" t="str">
+        <v>Mathematics</v>
+      </c>
+      <c r="G44" t="str">
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>13/9/2026, 8:33:57 pm</v>
+      </c>
+      <c r="B45">
+        <v>24</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Test Student</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Who is your study buddy?</v>
+      </c>
+      <c r="F45" t="str">
+        <v>Arun</v>
+      </c>
+      <c r="G45" t="str">
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>13/9/2026, 8:33:57 pm</v>
+      </c>
+      <c r="B46">
+        <v>24</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Test Student</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E46" t="str">
+        <v>Who would you call when you're having a bad day?</v>
+      </c>
+      <c r="F46" t="str">
+        <v>Karthik</v>
+      </c>
+      <c r="G46" t="str">
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>13/9/2026, 8:33:57 pm</v>
+      </c>
+      <c r="B47">
+        <v>24</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Test Student</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E47" t="str">
+        <v>Who do you text the most?</v>
+      </c>
+      <c r="F47" t="str">
+        <v>Arun</v>
+      </c>
+      <c r="G47" t="str">
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>13/9/2026, 8:33:57 pm</v>
+      </c>
+      <c r="B48">
+        <v>24</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Test Student</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E48" t="str">
+        <v>Who makes you laugh the most?</v>
+      </c>
+      <c r="F48" t="str">
+        <v>Karthik</v>
+      </c>
+      <c r="G48" t="str">
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>13/9/2026, 8:33:57 pm</v>
+      </c>
+      <c r="B49">
+        <v>24</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Test Student</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E49" t="str">
+        <v>Who is your best friend?</v>
+      </c>
+      <c r="F49" t="str">
+        <v>Arun</v>
+      </c>
+      <c r="G49" t="str">
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>13/9/2026, 8:33:19 pm</v>
+      </c>
+      <c r="B50">
+        <v>1</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Alex Mercer</v>
+      </c>
+      <c r="D50" t="str">
+        <v>AI Random Question</v>
+      </c>
+      <c r="E50" t="str">
+        <v>Which fictional character would you choose as your study partner? 🦸</v>
+      </c>
+      <c r="F50" t="str">
+        <v>Mathematics and Calculus</v>
+      </c>
+      <c r="G50" t="str">
+        <v>💀 Mathematics catching stray arrows as usual! We will conquer it together!</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>13/9/2026, 8:33:19 pm</v>
+      </c>
+      <c r="B51">
+        <v>1</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Alex Mercer</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E51" t="str">
+        <v>If your life were an anime/game/movie, what would its title be?</v>
+      </c>
+      <c r="F51" t="str">
+        <v>Solo Leveling: The Finals Arc ⚔️</v>
+      </c>
+      <c r="G51" t="str">
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>13/9/2026, 8:33:19 pm</v>
+      </c>
+      <c r="B52">
+        <v>1</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Alex Mercer</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E52" t="str">
+        <v>If you had a completely free day tomorrow, what would you do?</v>
+      </c>
+      <c r="F52" t="str">
+        <v>Sleep for 12 hours straight then binge anime 🍿</v>
+      </c>
+      <c r="G52" t="str">
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>13/9/2026, 8:33:19 pm</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Alex Mercer</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E53" t="str">
+        <v>What is the funniest thing that happened in your college life?</v>
+      </c>
+      <c r="F53" t="str">
+        <v>Professor caught us playing games in the front row 😂</v>
+      </c>
+      <c r="G53" t="str">
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>13/9/2026, 8:33:19 pm</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Alex Mercer</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E54" t="str">
+        <v>Who is your female best friend?</v>
+      </c>
+      <c r="F54" t="str">
+        <v>Priya</v>
+      </c>
+      <c r="G54" t="str">
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>13/9/2026, 8:33:19 pm</v>
+      </c>
+      <c r="B55">
+        <v>1</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Alex Mercer</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E55" t="str">
+        <v>Who is your male best friend?</v>
+      </c>
+      <c r="F55" t="str">
+        <v>Rahul</v>
+      </c>
+      <c r="G55" t="str">
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>13/9/2026, 8:33:19 pm</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Alex Mercer</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E56" t="str">
+        <v>Do you have a funny or secret nickname?</v>
+      </c>
+      <c r="F56" t="str">
+        <v>Rocky</v>
+      </c>
+      <c r="G56" t="str">
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>13/9/2026, 8:33:19 pm</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Alex Mercer</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E57" t="str">
+        <v>What's your favorite movie, anime, series, or game?</v>
+      </c>
+      <c r="F57" t="str">
+        <v>Interstellar</v>
+      </c>
+      <c r="G57" t="str">
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>13/9/2026, 8:33:19 pm</v>
+      </c>
+      <c r="B58">
+        <v>1</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Alex Mercer</v>
+      </c>
+      <c r="D58" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Which friend would survive an exam with you?</v>
+      </c>
+      <c r="F58" t="str">
+        <v>Arun</v>
+      </c>
+      <c r="G58" t="str">
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>13/9/2026, 8:33:19 pm</v>
+      </c>
+      <c r="B59">
+        <v>1</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Alex Mercer</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E59" t="str">
+        <v>What's your favorite way to relax?</v>
+      </c>
+      <c r="F59" t="str">
+        <v>🎮 Gaming, ▶️ YouTube</v>
+      </c>
+      <c r="G59" t="str">
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>13/9/2026, 8:33:19 pm</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Alex Mercer</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E60" t="str">
+        <v>Which subject is your biggest enemy?</v>
+      </c>
+      <c r="F60" t="str">
+        <v>Mathematics</v>
+      </c>
+      <c r="G60" t="str">
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>13/9/2026, 8:33:19 pm</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Alex Mercer</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E61" t="str">
+        <v>Who is your study buddy?</v>
+      </c>
+      <c r="F61" t="str">
+        <v>Arun</v>
+      </c>
+      <c r="G61" t="str">
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>13/9/2026, 8:33:19 pm</v>
+      </c>
+      <c r="B62">
+        <v>1</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Alex Mercer</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E62" t="str">
+        <v>Who would you call when you're having a bad day?</v>
+      </c>
+      <c r="F62" t="str">
+        <v>Karthik</v>
+      </c>
+      <c r="G62" t="str">
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>13/9/2026, 8:33:19 pm</v>
+      </c>
+      <c r="B63">
+        <v>1</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Alex Mercer</v>
+      </c>
+      <c r="D63" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E63" t="str">
+        <v>Who do you text the most?</v>
+      </c>
+      <c r="F63" t="str">
+        <v>Arun</v>
+      </c>
+      <c r="G63" t="str">
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>13/9/2026, 8:33:19 pm</v>
+      </c>
+      <c r="B64">
+        <v>1</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Alex Mercer</v>
+      </c>
+      <c r="D64" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E64" t="str">
+        <v>Who makes you laugh the most?</v>
+      </c>
+      <c r="F64" t="str">
+        <v>Karthik</v>
+      </c>
+      <c r="G64" t="str">
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>13/9/2026, 8:33:19 pm</v>
+      </c>
+      <c r="B65">
+        <v>1</v>
+      </c>
+      <c r="C65" t="str">
+        <v>Alex Mercer</v>
+      </c>
+      <c r="D65" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E65" t="str">
+        <v>Who is your best friend?</v>
+      </c>
+      <c r="F65" t="str">
+        <v>Arun</v>
+      </c>
+      <c r="G65" t="str">
+        <v>😂 Your core alliance is stacked with Rahul &amp; Priya anchoring your squad! Mathematics is officially the Final Boss on yo...</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>13/9/2026, 7:39:09 pm</v>
+      </c>
+      <c r="B66">
+        <v>1</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Alex Mercer</v>
+      </c>
+      <c r="D66" t="str">
+        <v>AI Random Question</v>
+      </c>
+      <c r="E66" t="str">
+        <v>What is your all-time most-used emoji during exam week? 🧐</v>
+      </c>
+      <c r="F66" t="str">
+        <v>Mathematics and Calculus</v>
+      </c>
+      <c r="G66" t="str">
+        <v>💀 Mathematics catching stray arrows as usual! We will conquer it together!</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>13/9/2026, 7:33:20 pm</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="str">
+        <v>Alex Mercer</v>
+      </c>
+      <c r="D67" t="str">
+        <v>AI Random Question</v>
+      </c>
+      <c r="E67" t="str">
+        <v>Which of your friends would secretly become a college professor? 👨‍🏫</v>
+      </c>
+      <c r="F67" t="str">
+        <v>Mathematics and Calculus</v>
+      </c>
+      <c r="G67" t="str">
+        <v>💀 Mathematics catching stray arrows as usual! We will conquer it together!</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>13/9/2026, 6:54:16 pm</v>
+      </c>
+      <c r="B68">
+        <v>1</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Alex Mercer</v>
+      </c>
+      <c r="D68" t="str">
+        <v>AI Random Question</v>
+      </c>
+      <c r="E68" t="str">
+        <v>If exams disappeared tomorrow, what would you do first? 😂</v>
+      </c>
+      <c r="F68" t="str">
+        <v>Mathematics and Calculus</v>
+      </c>
+      <c r="G68" t="str">
+        <v>💀 Mathematics catching stray arrows as usual! We will conquer it together!</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>13/9/2026, 6:53:31 pm</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Alex Mercer</v>
+      </c>
+      <c r="D69" t="str">
+        <v>AI Random Question</v>
+      </c>
+      <c r="E69" t="str">
+        <v>What is your all-time most-used emoji during exam week? 🧐</v>
+      </c>
+      <c r="F69" t="str">
+        <v>Mathematics and Calculus</v>
+      </c>
+      <c r="G69" t="str">
+        <v>💀 Mathematics catching stray arrows as usual! We will conquer it together!</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>13/9/2026, 6:53:17 pm</v>
+      </c>
+      <c r="B70">
+        <v>1</v>
+      </c>
+      <c r="C70" t="str">
+        <v>Alex Mercer</v>
+      </c>
+      <c r="D70" t="str">
+        <v>AI Random Question</v>
+      </c>
+      <c r="E70" t="str">
+        <v>What is your all-time most-used emoji during exam week? 🧐</v>
+      </c>
+      <c r="F70" t="str">
+        <v>Mathematics and Calculus</v>
+      </c>
+      <c r="G70" t="str">
+        <v>💀 Mathematics catching stray arrows as usual! We will conquer it together!</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>13/9/2026, 6:52:58 pm</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="str">
+        <v>Alex Mercer</v>
+      </c>
+      <c r="D71" t="str">
+        <v>AI Random Question</v>
+      </c>
+      <c r="E71" t="str">
+        <v>If exams disappeared tomorrow, what would you do first? 😂</v>
+      </c>
+      <c r="F71" t="str">
+        <v>Mathematics and Calculus</v>
+      </c>
+      <c r="G71" t="str">
+        <v>💀 Mathematics catching stray arrows as usual! We will conquer it together!</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>13/9/2026, 6:52:21 pm</v>
+      </c>
+      <c r="B72">
+        <v>1</v>
+      </c>
+      <c r="C72" t="str">
+        <v>Alex Mercer</v>
+      </c>
+      <c r="D72" t="str">
+        <v>AI Random Question</v>
+      </c>
+      <c r="E72" t="str">
+        <v>If exams disappeared tomorrow, what would you do first? 😂</v>
+      </c>
+      <c r="F72" t="str">
+        <v>Mathematics and Calculus</v>
+      </c>
+      <c r="G72" t="str">
+        <v>💀 Mathematics catching stray arrows as usual! We will conquer it together!</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>13/9/2026, 6:41:44 pm</v>
+      </c>
+      <c r="B73">
+        <v>5</v>
+      </c>
+      <c r="C73" t="str">
+        <v>praveen kumar</v>
+      </c>
+      <c r="D73" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E73" t="str">
+        <v>If your life were an anime/game/movie, what would its title be?</v>
+      </c>
+      <c r="F73" t="str">
+        <v>solo leveling</v>
+      </c>
+      <c r="G73" t="str">
+        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>13/9/2026, 6:41:44 pm</v>
+      </c>
+      <c r="B74">
+        <v>5</v>
+      </c>
+      <c r="C74" t="str">
+        <v>praveen kumar</v>
+      </c>
+      <c r="D74" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E74" t="str">
+        <v>If you had a completely free day tomorrow, what would you do?</v>
+      </c>
+      <c r="F74" t="str">
+        <v>non stop gaming</v>
+      </c>
+      <c r="G74" t="str">
+        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>13/9/2026, 6:41:44 pm</v>
+      </c>
+      <c r="B75">
+        <v>5</v>
+      </c>
+      <c r="C75" t="str">
+        <v>praveen kumar</v>
+      </c>
+      <c r="D75" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E75" t="str">
+        <v>What is the funniest thing that happened in your college life?</v>
+      </c>
+      <c r="F75" t="str">
+        <v>play find the importer</v>
+      </c>
+      <c r="G75" t="str">
+        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>13/9/2026, 6:41:44 pm</v>
+      </c>
+      <c r="B76">
+        <v>5</v>
+      </c>
+      <c r="C76" t="str">
+        <v>praveen kumar</v>
+      </c>
+      <c r="D76" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E76" t="str">
+        <v>Who is your female best friend?</v>
+      </c>
+      <c r="F76" t="str">
+        <v>pavithra</v>
+      </c>
+      <c r="G76" t="str">
+        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>13/9/2026, 6:41:44 pm</v>
+      </c>
+      <c r="B77">
+        <v>5</v>
+      </c>
+      <c r="C77" t="str">
+        <v>praveen kumar</v>
+      </c>
+      <c r="D77" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E77" t="str">
+        <v>Who is your male best friend?</v>
+      </c>
+      <c r="F77" t="str">
+        <v>rupesh</v>
+      </c>
+      <c r="G77" t="str">
+        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>13/9/2026, 6:41:44 pm</v>
+      </c>
+      <c r="B78">
+        <v>5</v>
+      </c>
+      <c r="C78" t="str">
+        <v>praveen kumar</v>
+      </c>
+      <c r="D78" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E78" t="str">
+        <v>Do you have a funny or secret nickname?</v>
+      </c>
+      <c r="F78" t="str">
+        <v>chapri</v>
+      </c>
+      <c r="G78" t="str">
+        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>13/9/2026, 6:41:44 pm</v>
+      </c>
+      <c r="B79">
+        <v>5</v>
+      </c>
+      <c r="C79" t="str">
+        <v>praveen kumar</v>
+      </c>
+      <c r="D79" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E79" t="str">
+        <v>What's your favorite movie, anime, series, or game?</v>
+      </c>
+      <c r="F79" t="str">
+        <v>attack on titan</v>
+      </c>
+      <c r="G79" t="str">
+        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>13/9/2026, 6:41:44 pm</v>
+      </c>
+      <c r="B80">
+        <v>5</v>
+      </c>
+      <c r="C80" t="str">
+        <v>praveen kumar</v>
+      </c>
+      <c r="D80" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E80" t="str">
+        <v>Which friend would survive an exam with you?</v>
+      </c>
+      <c r="F80" t="str">
+        <v>sanjay</v>
+      </c>
+      <c r="G80" t="str">
+        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>13/9/2026, 6:41:44 pm</v>
+      </c>
+      <c r="B81">
+        <v>5</v>
+      </c>
+      <c r="C81" t="str">
+        <v>praveen kumar</v>
+      </c>
+      <c r="D81" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E81" t="str">
+        <v>What's your favorite way to relax?</v>
+      </c>
+      <c r="F81" t="str">
+        <v>🎮 Gaming</v>
+      </c>
+      <c r="G81" t="str">
+        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>13/9/2026, 6:41:44 pm</v>
+      </c>
+      <c r="B82">
+        <v>5</v>
+      </c>
+      <c r="C82" t="str">
+        <v>praveen kumar</v>
+      </c>
+      <c r="D82" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E82" t="str">
+        <v>Which subject is your biggest enemy?</v>
+      </c>
+      <c r="F82" t="str">
+        <v>tamil</v>
+      </c>
+      <c r="G82" t="str">
+        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>13/9/2026, 6:41:44 pm</v>
+      </c>
+      <c r="B83">
+        <v>5</v>
+      </c>
+      <c r="C83" t="str">
+        <v>praveen kumar</v>
+      </c>
+      <c r="D83" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E83" t="str">
+        <v>Who is your study buddy?</v>
+      </c>
+      <c r="F83" t="str">
+        <v>sanjay</v>
+      </c>
+      <c r="G83" t="str">
+        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>13/9/2026, 6:41:44 pm</v>
+      </c>
+      <c r="B84">
+        <v>5</v>
+      </c>
+      <c r="C84" t="str">
+        <v>praveen kumar</v>
+      </c>
+      <c r="D84" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E84" t="str">
+        <v>Who would you call when you're having a bad day?</v>
+      </c>
+      <c r="F84" t="str">
+        <v>myself</v>
+      </c>
+      <c r="G84" t="str">
+        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>13/9/2026, 6:41:44 pm</v>
+      </c>
+      <c r="B85">
+        <v>5</v>
+      </c>
+      <c r="C85" t="str">
+        <v>praveen kumar</v>
+      </c>
+      <c r="D85" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E85" t="str">
+        <v>Who do you text the most?</v>
+      </c>
+      <c r="F85" t="str">
+        <v>pavithra</v>
+      </c>
+      <c r="G85" t="str">
+        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>13/9/2026, 6:41:44 pm</v>
+      </c>
+      <c r="B86">
+        <v>5</v>
+      </c>
+      <c r="C86" t="str">
+        <v>praveen kumar</v>
+      </c>
+      <c r="D86" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E86" t="str">
+        <v>Who makes you laugh the most?</v>
+      </c>
+      <c r="F86" t="str">
+        <v>pk</v>
+      </c>
+      <c r="G86" t="str">
+        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>13/9/2026, 6:41:44 pm</v>
+      </c>
+      <c r="B87">
+        <v>5</v>
+      </c>
+      <c r="C87" t="str">
+        <v>praveen kumar</v>
+      </c>
+      <c r="D87" t="str">
+        <v>Squad Check-Up</v>
+      </c>
+      <c r="E87" t="str">
+        <v>Who is your best friend?</v>
+      </c>
+      <c r="F87" t="str">
+        <v>sanjay</v>
+      </c>
+      <c r="G87" t="str">
+        <v>😂 Your core alliance is stacked with rupesh &amp; pavithra anchoring your squad! tamil is officially the Final Boss on your...</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>13/9/2026, 6:37:12 pm</v>
+      </c>
+      <c r="B88">
+        <v>1</v>
+      </c>
+      <c r="C88" t="str">
+        <v>Alex Mercer</v>
+      </c>
+      <c r="D88" t="str">
+        <v>AI Random Question</v>
+      </c>
+      <c r="E88" t="str">
+        <v>What is your most ridiculously productive time of day? ⏰</v>
+      </c>
+      <c r="F88" t="str">
+        <v>Mathematics and Calculus</v>
+      </c>
+      <c r="G88" t="str">
+        <v>💀 Mathematics catching stray arrows as usual! We will conquer it together!</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
         <v>13/9/2026, 6:36:31 pm</v>
       </c>
-      <c r="B40">
+      <c r="B89">
         <v>1</v>
       </c>
-      <c r="C40" t="str">
+      <c r="C89" t="str">
         <v>Alex Mercer</v>
       </c>
-      <c r="D40" t="str">
+      <c r="D89" t="str">
         <v>AI Random Question</v>
       </c>
-      <c r="E40" t="str">
+      <c r="E89" t="str">
         <v>Which fictional character would you choose as your study partner? 🦸</v>
       </c>
-      <c r="F40" t="str">
+      <c r="F89" t="str">
         <v>Mathematics and Calculus</v>
       </c>
-      <c r="G40" t="str">
+      <c r="G89" t="str">
         <v>💀 Mathematics catching stray arrows as usual! We will conquer it together!</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G40"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G89"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>